<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.002-04 La pomme de pin de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.002-04.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.002-04.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le cacao de la fenêtre</t>
+          <t>La pomme de pin de Nina</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>sentier de mousse, refuge de montagne, fenêtre de cacao</t>
+          <t>entrée, classe, goûter, puis maison</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, maman</t>
+          <t>Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut montrer sa pomme de pin et boire le cacao du refuge. Elle parle trop tôt. La vapeur et les voix couvrent. Elle lève la main, on l'entend.</t>
+          <t>Un filet d'escargot brille sur le mur. Sur une écaille, un éclat de mousse brille. Nina veut montrer la pomme de pin, maintenant. Elle tire trop vite : les mots se perdent. À la classe, elle ouvre la bouche trop tôt. Elle refuse de foncer, lève la main, attend, parle. Merci vécu. L'éclat de mousse tient sur l'écaille.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La mousse des sapins colle aux chaussures. L'air sent la résine froide. Une pomme de pin roule dans la poche. Elle chatouille les doigts, tout sec. Le refuge a une fenêtre allumée. Tu as vu la vapeur, Nina ? Ça sent le cacao. Je veux en boire. Et montrer ma pomme de pin. On va le dire, à la fenêtre. En ce moment, maman parle vers le bois. Sa voix se mêle à la vapeur. Nina a les mots tout prêts. Du cacao ! Et ma pomme de pin ! Les mots tombent dans la vapeur chaude. Personne ne se tourne. Deux tasses fument, trop loin. Maman. Maman parle encore, un gant sur le rebord. Nina ferme la bouche. Elle lève la main, tout droit. La pomme de pin est dans l'autre main. Sa main reste en l'air, près de la vitre. La vapeur s'écarte un peu. Maman se tourne. Tu voulais dire quelque chose ? Du cacao. Et ça, pour le rebord. Je t'entends, maintenant. Une tasse chaude arrive, toute ronde. Nina pose la pomme de pin sur le bois. Elle ressemble à un hérisson. Merci, Nina. Tu as attendu, et je t'ai entendue. Le cacao brûle un peu la lèvre. Il sent le bois et le lait. On souffle ensemble ? Fffff.</t>
+          <t>Un filet d'escargot brille sur le mur. Il est argenté, un peu visqueux. L'air sent la mousse froide. Nina connaît ce mur de l'entrée. Ce filet, lui, est nouveau. Une pomme de pin roule dans la poche. Elle chatouille les doigts, sèche. Sur une écaille, un éclat de mousse brille. Il est vert, maman. C'est la mousse du sentier. Le cartable est un peu humide, dehors. Maman tient le cartable de Nina. Le tissu sent la pluie et le bois. Je veux montrer la pomme de pin, maintenant ! Près du hérisson. La pomme verte est pour le goûter. Papa parle près du cartable, une main sur le tissu. Je la sors ! Nina tire trop vite. La pomme de pin glisse, presque. Les mots se cognent à ceux de papa. Personne ne tourne la tête. Oh. L'éclat de mousse tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux la montrer ? Oui, papa. Tu vas t'asseoir sur le tapis ? D'accord, maman. En ce moment, Nina entre dans la classe. Au revoir, Nina. Au revoir, maman. Nina s'assoit sur le tapis. Le tapis est un peu froid, sous les genoux. La pomme de pin reste dans la poche. Près du tableau, la maîtresse montre une affiche. C'est un hérisson. Les piquants sont dessinés au crayon brun. La classe écoute l'affiche. Nina a une idée. Les piquants ressemblent à la pomme de pin. Je veux parler des piquants.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La mousse des sapins colle aux chaussures. L'air sent la résine froide. Une pomme de pin roule dans la poche. Elle chatouille les doigts, tout sec. Le refuge a une fenêtre allumée. Tu as vu la vapeur, Nina ? Ça sent le cacao. Je veux en boire. Et montrer ma pomme de pin. On va le dire, à la fenêtre. En ce moment, maman parle vers le bois. Sa voix se mêle à la vapeur. Nina a les mots tout prêts. Du cacao ! Et ma pomme de pin ! Les mots tombent dans la vapeur chaude. Personne ne se tourne. Deux tasses fument, trop loin. Maman. Maman parle encore, un gant sur le rebord. Nina ferme la bouche. Elle lève la main, tout droit. La pomme de pin est dans l'autre main. Sa main reste en l'air, près de la vitre. La vapeur s'écarte un peu. Maman se tourne. Tu voulais dire quelque chose ? Du cacao. Et ça, pour le rebord. Je t'entends, maintenant. Une tasse chaude arrive, toute ronde. Nina pose la pomme de pin sur le bois. Elle ressemble à un hérisson. Merci, Nina. Tu as attendu, et je t'ai entendue. Le cacao brûle un peu la lèvre. Il sent le bois et le lait. On souffle ensemble ? Fffff.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un filet d'escargot brille sur le mur. Il est argenté, un peu visqueux. L'air sent la mousse froide. Nina connaît ce mur de l'entrée. Ce filet, lui, est nouveau. Une pomme de pin roule dans la poche. Elle chatouille les doigts, sèche. Sur une écaille, un &lt;emphasis level="moderate"&gt;éclat de mousse&lt;/emphasis&gt; brille. Il est vert, maman. C'est la mousse du sentier. Le cartable est un peu humide, dehors. Maman tient le cartable de Nina. Le tissu sent la pluie et le bois. Je veux montrer la pomme de pin, maintenant ! Près du hérisson. La pomme verte est pour le goûter. Papa parle près du cartable, une main sur le tissu. Je la sors ! Nina tire trop vite. La pomme de pin glisse, presque. Les mots se cognent à ceux de papa. Personne ne tourne la tête. Oh. L'éclat de mousse tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux la montrer ? Oui, papa. Tu vas t'asseoir sur le tapis ? D'accord, maman. En ce moment, Nina entre dans la classe. Au revoir, Nina. Au revoir, maman. Nina s'assoit sur le tapis. Le tapis est un peu froid, sous les genoux. La pomme de pin reste dans la poche. Près du tableau, la maîtresse montre une affiche. C'est un hérisson. Les piquants sont dessinés au crayon brun. La classe écoute l'affiche. Nina a une idée. Les piquants ressemblent à la pomme de pin. Je veux parler des piquants.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Idris arrive en classe avec maman. Maman dit au revoir. Idris s'assoit sur le tapis. La maîtresse pose une question. Idris a une idée. Il lève la main. Il faut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Un camarade parle d'abord. Idris attend encore. Puis la maîtresse dit : Idris, c'est ton tour. Idris parle. Il dit : le hérisson a des piquants. La maîtresse sourit. Plus tard, c'est le goûter. Idris a envie de raconter son goûter. Il lève la main. Il faut attendre. Une camarade parle. Idris attend. Puis la maîtresse dit : Idris. Idris parle. Il dit : j'ai une pomme. Sur le tapis, puis au goûter, c'est pareil. On lève la main. Il faut attendre. Puis parler. Le soir, maman demande. Idris dit : j'ai levé la main. J'ai su attendre. Puis j'ai parlé. Maman dit merci. Idris range son cartable. [pause]</t>
+          <t>Un filet d'escargot brille sur le mur. Il est argenté, un peu visqueux. L'air sent la mousse froide. Nina connaît ce mur de l'entrée. Ce filet, lui, est nouveau. Une pomme de pin roule dans la poche. Elle chatouille les doigts, sèche. Sur une écaille, un &lt;emphasis&gt;éclat de mousse&lt;/emphasis&gt; brille. Il est vert, maman. C'est la mousse du sentier. Le cartable est un peu humide, dehors. Maman tient le cartable de Nina. Le tissu sent la pluie et le bois. Je veux montrer la pomme de pin, maintenant ! Près du hérisson. La pomme verte est pour le goûter. Papa parle près du cartable, une main sur le tissu. Je la sors ! Nina tire trop vite. La pomme de pin glisse, presque. Les mots se cognent à ceux de papa. Personne ne tourne la tête. Oh. L'éclat de mousse tremble, puis tient. Le sourire de Nina disparaît. Dans sa poitrine, envie et inquiétude se bousculent. Ça ne veut pas. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu veux la montrer ? Oui, papa. Tu vas t'asseoir sur le tapis ? D'accord, maman. En ce moment, Nina entre dans la classe. Au revoir, Nina. Au revoir, maman. Nina s'assoit sur le tapis. Le tapis est un peu froid, sous les genoux. La pomme de pin reste dans la poche. Près du tableau, la maîtresse montre une affiche. C'est un hérisson. Les piquants sont dessinés au crayon brun. La classe écoute l'affiche. Nina a une idée. Les piquants ressemblent à la pomme de pin. Je veux parler des piquants. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de mousse</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,48 +1326,59 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_montrer_la_pomme_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La mousse des sapins colle aux chaussures.
-narrateur|L'air sent la résine froide.
+          <t>narrateur|Un filet d'escargot brille sur le mur.
+narrateur|Il est argenté, un peu visqueux.
+narrateur|L'air sent la mousse froide.
+narrateur|Nina connaît ce mur de l'entrée.
+narrateur|Ce filet, lui, est nouveau.
 narrateur|Une pomme de pin roule dans la poche.
-narrateur|Elle chatouille les doigts, tout sec.
-narrateur|Le refuge a une fenêtre allumée.
-maman|Tu as vu la vapeur, Nina ?
-enfant-f|Ça sent le cacao.
-enfant-f|Je veux en boire.
-enfant-f|Et montrer ma pomme de pin.
-maman|On va le dire, à la fenêtre.
-narrateur|En ce moment, maman parle vers le bois.
-narrateur|Sa voix se mêle à la vapeur.
-narrateur|Nina a les mots tout prêts.
-enfant-f|Du cacao !
-enfant-f|Et ma pomme de pin !
-narrateur|Les mots tombent dans la vapeur chaude.
-narrateur|Personne ne se tourne.
-narrateur|Deux tasses fument, trop loin.
-enfant-f|Maman.
-narrateur|Maman parle encore, un gant sur le rebord.
-narrateur|Nina ferme la bouche.
-narrateur|Elle lève la main, tout droit.
-narrateur|La pomme de pin est dans l'autre main.
-narrateur|Sa main reste en l'air, près de la vitre.
-narrateur|La vapeur s'écarte un peu.
-narrateur|Maman se tourne.
-maman|Tu voulais dire quelque chose ?
-enfant-f|Du cacao.
-enfant-f|Et ça, pour le rebord.
-maman|Je t'entends, maintenant.
-narrateur|Une tasse chaude arrive, toute ronde.
-narrateur|Nina pose la pomme de pin sur le bois.
-enfant-f|Elle ressemble à un hérisson.
-maman|Merci, Nina.
-maman|Tu as attendu, et je t'ai entendue.
-narrateur|Le cacao brûle un peu la lèvre.
-narrateur|Il sent le bois et le lait.
-maman|On souffle ensemble ?
-enfant-f|Fffff.</t>
+narrateur|Elle chatouille les doigts, sèche.
+narrateur|Sur une écaille, un éclat de mousse brille.
+enfant-f|Il est vert, maman.
+maman|C'est la mousse du sentier.
+papa|Le cartable est un peu humide, dehors.
+narrateur|Maman tient le cartable de Nina.
+narrateur|Le tissu sent la pluie et le bois.
+enfant-f|Je veux montrer la pomme de pin, maintenant !
+enfant-f|Près du hérisson.
+papa|La pomme verte est pour le goûter.
+narrateur|Papa parle près du cartable, une main sur le tissu.
+enfant-f|Je la sors !
+narrateur|Nina tire trop vite.
+narrateur|La pomme de pin glisse, presque.
+narrateur|Les mots se cognent à ceux de papa.
+narrateur|Personne ne tourne la tête.
+enfant-f|Oh.
+narrateur|L'éclat de mousse tremble, puis tient.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, envie et inquiétude se bousculent.
+enfant-f|Ça ne veut pas.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu veux la montrer ?
+enfant-f|Oui, papa.
+maman|Tu vas t'asseoir sur le tapis ?
+enfant-f|D'accord, maman.
+narrateur|En ce moment, Nina entre dans la classe.
+maman|Au revoir, Nina.
+enfant-f|Au revoir, maman.
+narrateur|Nina s'assoit sur le tapis.
+narrateur|Le tapis est un peu froid, sous les genoux.
+narrateur|La pomme de pin reste dans la poche.
+narrateur|Près du tableau, la maîtresse montre une affiche.
+narrateur|C'est un hérisson.
+narrateur|Les piquants sont dessinés au crayon brun.
+narrateur|La classe écoute l'affiche.
+narrateur|Nina a une idée.
+narrateur|Les piquants ressemblent à la pomme de pin.
+enfant-f|Je veux parler des piquants.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1404,12 +1415,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nina veut parler. Que fait-elle d'abord ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nina veut &lt;emphasis level="moderate"&gt;parler&lt;/emphasis&gt;. Que fait-elle d'abord ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Idris veut parler. Que fait-il d'abord ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nina veut &lt;emphasis&gt;parler&lt;/emphasis&gt;. Que fait-elle d'abord ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1434,7 +1445,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Personne ne l'entend. Que fait Nina d'abord ?</t>
+          <t>Elle lève la main et elle attend. Que fait Nina ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1472,7 +1483,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1480,10 +1491,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1498,34 +1509,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>parler</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1534,23 +1549,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_attend_puis_parle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1583,17 +1598,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>La pomme de pin sèche sur le rebord. Nina souffle encore sur la tasse. Un nuage court sur le cacao. Il est moins chaud. Tu goûtes ? Oui. Une moustache brune reste au-dessus de la lèvre. Tu m'as entendue. Oui. Quand la vapeur s'est écartée. Quand ta main était là. Un grelot tinte, plus bas sur le sentier. La mousse brille encore aux chaussures. Ta pomme de pin tient bien ? Sur le bois, oui. Nina la tourne d'un doigt. Les écailles font un tout petit bruit. On la reprend, après ? Dans la poche.</t>
+          <t>Nina ouvre la bouche trop vite. Les piquants, comme ma pomme de pin ! Un camarade parle, près de l'affiche. Le hérisson a des piquants. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Elle lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Nina attend que le silence arrive. Sur l'écaille, l'éclat de mousse brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Le hérisson a des piquants. Comme ma pomme de pin. Elle la pose près de l'affiche. Les piquants et les écailles se regardent. Plus tard, c'est le goûter. Les boîtes s'ouvrent. Ça sent la pomme verte. Nina a envie de raconter son goûter. J'ai une pomme ! Les voix se mélangent, près des boîtes. Nina referme la bouche. Elle lève la main. Elle attend. Une boîte se ferme, un peu plus loin. J'ai une pomme verte. Le soir, la porte s'ouvre. Te voilà, Nina. Le manteau sent la mousse. Nina pose le cartable contre le mur. J'ai montré la pomme de pin. Les piquants, comme les écailles. Merci, Nina. Papa a entendu toute la phrase. Tu veux ta pomme ? Oui, maman. Le ventre de Nina se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>La pomme de pin sèche sur le rebord. Nina souffle encore sur la tasse. Un nuage court sur le cacao. Il est moins chaud. Tu goûtes ? Oui. Une moustache brune reste au-dessus de la lèvre. Tu m'as entendue. Oui. Quand la vapeur s'est écartée. Quand ta main était là. Un grelot tinte, plus bas sur le sentier. La mousse brille encore aux chaussures. Ta pomme de pin tient bien ? Sur le bois, oui. Nina la tourne d'un doigt. Les écailles font un tout petit bruit. On la reprend, après ? Dans la poche.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina ouvre la bouche trop vite. Les piquants, comme ma pomme de pin ! Un camarade parle, près de l'affiche. Le hérisson a des piquants. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Elle lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Nina attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Sur l'écaille, l'éclat de mousse brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Le hérisson a des piquants. Comme ma pomme de pin. Elle la pose près de l'affiche. Les piquants et les écailles se regardent. Plus tard, c'est le goûter. Les boîtes s'ouvrent. Ça sent la pomme verte. Nina a envie de raconter son goûter. J'ai une pomme ! Les voix se mélangent, près des boîtes. Nina referme la bouche. Elle lève la main. Elle attend. Une boîte se ferme, un peu plus loin. J'ai une pomme verte. Le soir, la porte s'ouvre. Te voilà, Nina. Le manteau sent la mousse. Nina pose le cartable contre le mur. J'ai montré la pomme de pin. Les piquants, comme les écailles. Merci, Nina. Papa a entendu toute la phrase. Tu veux ta pomme ? Oui, maman. Le ventre de Nina se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Idris a levé la main. Il a attendu. &lt;emphasis&gt;puis&lt;/emphasis&gt; il a parlé. C'était son tour. [pause]</t>
+          <t>Nina ouvre la bouche trop vite. Les piquants, comme ma pomme de pin ! Un camarade parle, près de l'affiche. Le hérisson a des piquants. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Elle lève la main, près du tapis. Sa main reste en l'air. Le camarade finit sa phrase. Nina attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Sur l'écaille, l'éclat de mousse brille. Je peux dire quelque chose ? La classe tourne un peu la tête. Le hérisson a des piquants. Comme ma pomme de pin. Elle la pose près de l'affiche. Les piquants et les écailles se regardent. Plus tard, c'est le goûter. Les boîtes s'ouvrent. Ça sent la pomme verte. Nina a envie de raconter son goûter. J'ai une pomme ! Les voix se mélangent, près des boîtes. Nina referme la bouche. Elle lève la main. Elle attend. Une boîte se ferme, un peu plus loin. J'ai une pomme verte. Le soir, la porte s'ouvre. Te voilà, Nina. Le manteau sent la mousse. Nina pose le cartable contre le mur. J'ai montré la pomme de pin. Les piquants, comme les écailles. Merci, Nina. Papa a entendu toute la phrase. Tu veux ta pomme ? Oui, maman. Le ventre de Nina se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1640,7 +1655,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1648,10 +1663,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1674,30 +1689,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>puis</t>
+          <t>silence</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1706,10 +1721,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1722,30 +1737,53 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|La pomme de pin sèche sur le rebord.
-narrateur|Nina souffle encore sur la tasse.
-narrateur|Un nuage court sur le cacao.
-enfant-f|Il est moins chaud.
-maman|Tu goûtes ?
-enfant-f|Oui.
-narrateur|Une moustache brune reste au-dessus de la lèvre.
-enfant-f|Tu m'as entendue.
-maman|Oui.
-maman|Quand la vapeur s'est écartée.
-maman|Quand ta main était là.
-narrateur|Un grelot tinte, plus bas sur le sentier.
-narrateur|La mousse brille encore aux chaussures.
-maman|Ta pomme de pin tient bien ?
-enfant-f|Sur le bois, oui.
-narrateur|Nina la tourne d'un doigt.
-narrateur|Les écailles font un tout petit bruit.
-maman|On la reprend, après ?
-enfant-f|Dans la poche.</t>
+          <t>narrateur|Nina ouvre la bouche trop vite.
+enfant-f|Les piquants, comme ma pomme de pin !
+narrateur|Un camarade parle, près de l'affiche.
+copain|Le hérisson a des piquants.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Elle lève la main, près du tapis.
+narrateur|Sa main reste en l'air.
+narrateur|Le camarade finit sa phrase.
+narrateur|Nina attend que le silence arrive.
+narrateur|Sur l'écaille, l'éclat de mousse brille.
+enfant-f|Je peux dire quelque chose ?
+narrateur|La classe tourne un peu la tête.
+enfant-f|Le hérisson a des piquants.
+enfant-f|Comme ma pomme de pin.
+narrateur|Elle la pose près de l'affiche.
+narrateur|Les piquants et les écailles se regardent.
+narrateur|Plus tard, c'est le goûter.
+narrateur|Les boîtes s'ouvrent.
+narrateur|Ça sent la pomme verte.
+narrateur|Nina a envie de raconter son goûter.
+enfant-f|J'ai une pomme !
+narrateur|Les voix se mélangent, près des boîtes.
+narrateur|Nina referme la bouche.
+narrateur|Elle lève la main.
+narrateur|Elle attend.
+narrateur|Une boîte se ferme, un peu plus loin.
+enfant-f|J'ai une pomme verte.
+narrateur|Le soir, la porte s'ouvre.
+maman|Te voilà, Nina.
+papa|Le manteau sent la mousse.
+narrateur|Nina pose le cartable contre le mur.
+enfant-f|J'ai montré la pomme de pin.
+enfant-f|Les piquants, comme les écailles.
+papa|Merci, Nina.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu veux ta pomme ?
+enfant-f|Oui, maman.
+narrateur|Le ventre de Nina se desserre.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1777,17 +1815,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>La tasse est vide, encore chaude. Nina reprend la pomme de pin. On redescend ? Oui. J'ai bu le cacao. Oui. Je t'ai entendue. Le sentier sent la mousse et le lait. La fenêtre reste allumée, plus loin. Elle est bien dans la poche ? Elle chatouille encore.</t>
+          <t>Nina veut tout dire, d'un coup. Elle prend la pomme et la pomme de pin. La pomme verte glisse vers le sol. La pomme de pin roule vers le rebord. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde la pomme de pin. Elle écoute l'entrée, un instant. Le filet d'escargot sèche un peu, sur le mur. Sur le rebord, l'éclat de mousse brille. Comme ce matin ! Tu le vois, toi ? Oui, sur cette écaille. Nina pose la pomme de pin, d'abord. Puis elle rattrape la pomme verte. La pomme, Nina ? Oui. Elle s'assoit. La pomme est lisse, un peu froide. Elle croque. Le jus est doux.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>La tasse est vide, encore chaude. Nina reprend la pomme de pin. On redescend ? Oui. J'ai bu le cacao. Oui. Je t'ai entendue. Le sentier sent la mousse et le lait. La fenêtre reste allumée, plus loin. Elle est bien dans la poche ? Elle chatouille encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina veut tout dire, d'un coup. Elle prend la pomme et la pomme de pin. La pomme verte glisse vers le sol. La pomme de pin roule vers le rebord. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde la pomme de pin. Elle écoute l'entrée, un instant. Le filet d'escargot sèche un peu, sur le mur. Sur le rebord, l'&lt;emphasis level="moderate"&gt;éclat de mousse&lt;/emphasis&gt; brille. Comme ce matin ! Tu le vois, toi ? Oui, sur cette écaille. Nina pose la pomme de pin, d'abord. Puis elle rattrape la pomme verte. La pomme, Nina ? Oui. Elle s'assoit. La pomme est lisse, un peu froide. Elle croque. Le jus est doux.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Idris met son manteau. Maman l'attend à la porte. [pause]</t>
+          <t>&lt;low-pitch&gt;Nina veut tout dire, d'un coup. Elle prend la pomme et la pomme de pin. La pomme verte glisse vers le sol. La pomme de pin roule vers le rebord. Ça tombe ! Nina veut foncer, d'un coup. Nina refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Elle regarde la pomme de pin. Elle écoute l'entrée, un instant. Le filet d'escargot sèche un peu, sur le mur. Sur le rebord, l'&lt;emphasis&gt;éclat de mousse&lt;/emphasis&gt; brille. Comme ce matin ! Tu le vois, toi ? Oui, sur cette écaille. Nina pose la pomme de pin, d'abord. Puis elle rattrape la pomme verte. La pomme, Nina ? Oui. Elle s'assoit. La pomme est lisse, un peu froide. Elle croque. Le jus est doux.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,7 +1872,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1842,22 +1880,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1866,28 +1908,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de mousse</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,39 +1942,57 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|La tasse est vide, encore chaude.
-narrateur|Nina reprend la pomme de pin.
-maman|On redescend ?
+          <t>narrateur|Nina veut tout dire, d'un coup.
+narrateur|Elle prend la pomme et la pomme de pin.
+narrateur|La pomme verte glisse vers le sol.
+narrateur|La pomme de pin roule vers le rebord.
+enfant-f|Ça tombe !
+narrateur|Nina veut foncer, d'un coup.
+narrateur|Nina refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Elle regarde la pomme de pin.
+narrateur|Elle écoute l'entrée, un instant.
+narrateur|Le filet d'escargot sèche un peu, sur le mur.
+narrateur|Sur le rebord, l'éclat de mousse brille.
+enfant-f|Comme ce matin !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur cette écaille.
+narrateur|Nina pose la pomme de pin, d'abord.
+narrateur|Puis elle rattrape la pomme verte.
+maman|La pomme, Nina ?
 enfant-f|Oui.
-enfant-f|J'ai bu le cacao.
-maman|Oui.
-maman|Je t'ai entendue.
-narrateur|Le sentier sent la mousse et le lait.
-narrateur|La fenêtre reste allumée, plus loin.
-maman|Elle est bien dans la poche ?
-enfant-f|Elle chatouille encore.</t>
+narrateur|Elle s'assoit.
+narrateur|La pomme est lisse, un peu froide.
+narrateur|Elle croque.
+narrateur|Le jus est doux.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte,manteau</t>
+          <t>pomme,rebord</t>
         </is>
       </c>
     </row>
@@ -1955,17 +2019,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La pomme de pin chatouille la poche. Tu m'as entendue. Oui. Une moustache de cacao sèche un peu. Les sapins sentent encore la résine.</t>
+          <t>La pomme de pin attend sur le rebord. Le filet d'escargot sèche sur le mur. L'éclat est là, papa. Tu le vois sur l'écaille ? Oui, papa. On est bien, ici. La pomme verte repose près de la fenêtre. La fenêtre tremble moins. On m'a entendue. On t'a entendue, Nina. Oui, maman. Nina pose la joue près des écailles. Les écailles sont sèches, un peu rudes. C'est froid. Dehors, la mousse reste sur le sentier. L'éclat de mousse tient sur l'écaille.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La pomme de pin chatouille la poche. Tu m'as entendue. Oui. Une moustache de cacao sèche un peu. Les sapins sentent encore la résine.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La pomme de pin attend sur le rebord. Le filet d'escargot sèche sur le mur. L'éclat est là, papa. Tu le vois sur l'écaille ? Oui, papa. On est bien, ici. La pomme verte repose près de la fenêtre. La fenêtre tremble moins. On m'a entendue. On t'a entendue, Nina. Oui, maman. Nina pose la joue près des écailles. Les écailles sont sèches, un peu rudes. C'est froid. Dehors, la mousse reste sur le sentier. L'&lt;emphasis level="moderate"&gt;éclat de mousse&lt;/emphasis&gt; tient sur l'écaille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La pomme de pin attend sur le rebord. Le filet d'escargot sèche sur le mur. L'éclat est là, papa. Tu le vois sur l'écaille ? Oui, papa. On est bien, ici. La pomme verte repose près de la fenêtre. La fenêtre tremble moins. On m'a entendue. On t'a entendue, Nina. Oui, maman. Nina pose la joue près des écailles. Les écailles sont sèches, un peu rudes. C'est froid. Dehors, la mousse reste sur le sentier. L'&lt;emphasis&gt;éclat de mousse&lt;/emphasis&gt; tient sur l'écaille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2012,18 +2076,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2032,12 +2096,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2046,17 +2110,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de mousse</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2065,11 +2133,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2078,28 +2146,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_l_ecaille; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La pomme de pin chatouille la poche.
-enfant-f|Tu m'as entendue.
-maman|Oui.
-narrateur|Une moustache de cacao sèche un peu.
-narrateur|Les sapins sentent encore la résine.</t>
+          <t>narrateur|La pomme de pin attend sur le rebord.
+narrateur|Le filet d'escargot sèche sur le mur.
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur l'écaille ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|La pomme verte repose près de la fenêtre.
+narrateur|La fenêtre tremble moins.
+enfant-f|On m'a entendue.
+maman|On t'a entendue, Nina.
+enfant-f|Oui, maman.
+narrateur|Nina pose la joue près des écailles.
+narrateur|Les écailles sont sèches, un peu rudes.
+enfant-f|C'est froid.
+narrateur|Dehors, la mousse reste sur le sentier.
+narrateur|L'éclat de mousse tient sur l'écaille.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>rebord,mousse</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2212,6 +2300,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>